<commit_message>
RP-635: read cells as stored, not as shown (RP-631's owner)
Pins the decision in a test: 12 formatted 0000 reads 12, 0012 typed as text reads 0012.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/test/fixtures/registers/formats.xlsx
+++ b/apps/api/test/fixtures/registers/formats.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,20 +467,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.15</v>
+          <t>0012</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>0012</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>12345678901234567890</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>12345678901234567890</t>
         </is>

</xml_diff>